<commit_message>
Add PDEA most wanted watchlist with reusable image and PDF OCR support
</commit_message>
<xml_diff>
--- a/data/rules/pickLists.xlsx
+++ b/data/rules/pickLists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA13435-3199-4011-BEE0-167F26CF8BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0975A12-D7E9-4025-A626-A14A3E5D7123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="1100" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pick Lists" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2133" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="759">
   <si>
     <t>Path</t>
   </si>
@@ -2288,13 +2288,25 @@
   </si>
   <si>
     <t>People Involved</t>
+  </si>
+  <si>
+    <t>PDEA</t>
+  </si>
+  <si>
+    <t>Philippine Drug Enforcement Agency.</t>
+  </si>
+  <si>
+    <t>PDEA_MOST_WANTED</t>
+  </si>
+  <si>
+    <t>Most Wanted poster published by PDEA.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2329,6 +2341,12 @@
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF202B3B"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -2475,7 +2493,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2526,6 +2544,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -33412,8 +33433,36 @@
         <v>746</v>
       </c>
     </row>
-    <row r="1021" spans="1:5" s="4" customFormat="1" ht="12.5"/>
-    <row r="1022" spans="1:5" s="4" customFormat="1" ht="12.5"/>
+    <row r="1021" spans="1:5" ht="15" customHeight="1">
+      <c r="A1021" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1021" s="18" t="s">
+        <v>755</v>
+      </c>
+      <c r="C1021" s="18"/>
+      <c r="D1021" s="18"/>
+      <c r="E1021" s="18" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:5" ht="15" customHeight="1">
+      <c r="A1022" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1022" s="18" t="s">
+        <v>757</v>
+      </c>
+      <c r="C1022" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1022" s="18" t="s">
+        <v>755</v>
+      </c>
+      <c r="E1022" s="18" t="s">
+        <v>758</v>
+      </c>
+    </row>
     <row r="1023" spans="1:5" s="4" customFormat="1" ht="12.5"/>
     <row r="1024" spans="1:5" s="4" customFormat="1" ht="12.5"/>
     <row r="1025" spans="1:5" ht="12.5">

</xml_diff>

<commit_message>
Add PNP SDSPPO most wanted source with embedded image OCR
</commit_message>
<xml_diff>
--- a/data/rules/pickLists.xlsx
+++ b/data/rules/pickLists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0975A12-D7E9-4025-A626-A14A3E5D7123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593DFC11-832D-41A5-8F9D-6672EE9B2B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="13550" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pick Lists" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2167" uniqueCount="774">
   <si>
     <t>Path</t>
   </si>
@@ -2300,6 +2300,51 @@
   </si>
   <si>
     <t>Most Wanted poster published by PDEA.</t>
+  </si>
+  <si>
+    <t>PNP</t>
+  </si>
+  <si>
+    <t>Philippine National Police.</t>
+  </si>
+  <si>
+    <t>PNP_SDSPPO_MOST_WANTED</t>
+  </si>
+  <si>
+    <t>Reward posters published on the PNP SDSPPO Most Wanted Persons page.</t>
+  </si>
+  <si>
+    <t>Reward amount as printed. Currency and current availability are not inferred.</t>
+  </si>
+  <si>
+    <t>Joint Order Number</t>
+  </si>
+  <si>
+    <t>DND-DILG joint order reference from the JOR NO. field. It may be shared across persons.</t>
+  </si>
+  <si>
+    <t>Region as Listed</t>
+  </si>
+  <si>
+    <t>Region label as printed by the source. It is not a residence or nationality.</t>
+  </si>
+  <si>
+    <t>Position as Listed</t>
+  </si>
+  <si>
+    <t>Position or role described by the source, potentially historical. It is not asserted as current employment.</t>
+  </si>
+  <si>
+    <t>Case Reference</t>
+  </si>
+  <si>
+    <t>Court or case reference text as printed. It is not a unique person identifier.</t>
+  </si>
+  <si>
+    <t>Issuing Court</t>
+  </si>
+  <si>
+    <t>Issuing court text transcribed from the source. It is not a personal address.</t>
   </si>
 </sst>
 </file>
@@ -33463,56 +33508,120 @@
         <v>758</v>
       </c>
     </row>
-    <row r="1023" spans="1:5" s="4" customFormat="1" ht="12.5"/>
-    <row r="1024" spans="1:5" s="4" customFormat="1" ht="12.5"/>
-    <row r="1025" spans="1:5" ht="12.5">
-      <c r="A1025" s="4"/>
-      <c r="B1025" s="4"/>
-      <c r="C1025" s="4"/>
-      <c r="D1025" s="6"/>
-      <c r="E1025" s="4"/>
-    </row>
-    <row r="1026" spans="1:5" ht="12.5">
-      <c r="A1026" s="4"/>
-      <c r="B1026" s="4"/>
-      <c r="C1026" s="4"/>
-      <c r="D1026" s="6"/>
-      <c r="E1026" s="4"/>
-    </row>
-    <row r="1027" spans="1:5" ht="12.5">
-      <c r="A1027" s="4"/>
-      <c r="B1027" s="4"/>
-      <c r="C1027" s="4"/>
-      <c r="D1027" s="6"/>
-      <c r="E1027" s="4"/>
-    </row>
-    <row r="1028" spans="1:5" ht="12.5">
-      <c r="A1028" s="4"/>
-      <c r="B1028" s="4"/>
-      <c r="C1028" s="4"/>
-      <c r="D1028" s="6"/>
-      <c r="E1028" s="4"/>
-    </row>
-    <row r="1029" spans="1:5" ht="12.5">
-      <c r="A1029" s="4"/>
-      <c r="B1029" s="4"/>
-      <c r="C1029" s="4"/>
-      <c r="D1029" s="6"/>
-      <c r="E1029" s="4"/>
-    </row>
-    <row r="1030" spans="1:5" ht="12.5">
-      <c r="A1030" s="4"/>
-      <c r="B1030" s="4"/>
-      <c r="C1030" s="4"/>
-      <c r="D1030" s="6"/>
-      <c r="E1030" s="4"/>
-    </row>
-    <row r="1031" spans="1:5" ht="12.5">
-      <c r="A1031" s="4"/>
-      <c r="B1031" s="4"/>
-      <c r="C1031" s="4"/>
-      <c r="D1031" s="6"/>
-      <c r="E1031" s="4"/>
+    <row r="1023" spans="1:5" ht="15" customHeight="1">
+      <c r="A1023" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1023" s="18" t="s">
+        <v>759</v>
+      </c>
+      <c r="C1023" s="18"/>
+      <c r="D1023" s="18"/>
+      <c r="E1023" s="18" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:5" ht="15" customHeight="1">
+      <c r="A1024" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1024" s="18" t="s">
+        <v>761</v>
+      </c>
+      <c r="C1024" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1024" s="18" t="s">
+        <v>759</v>
+      </c>
+      <c r="E1024" s="18" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:5" ht="15" customHeight="1">
+      <c r="A1025" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1025" s="18" t="s">
+        <v>627</v>
+      </c>
+      <c r="C1025" s="18"/>
+      <c r="D1025" s="18"/>
+      <c r="E1025" s="18" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:5" ht="15" customHeight="1">
+      <c r="A1026" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1026" s="18" t="s">
+        <v>764</v>
+      </c>
+      <c r="C1026" s="18"/>
+      <c r="D1026" s="18"/>
+      <c r="E1026" s="18" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:5" ht="15" customHeight="1">
+      <c r="A1027" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1027" s="18" t="s">
+        <v>766</v>
+      </c>
+      <c r="C1027" s="18"/>
+      <c r="D1027" s="18"/>
+      <c r="E1027" s="18" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:5" ht="15" customHeight="1">
+      <c r="A1028" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1028" s="18" t="s">
+        <v>768</v>
+      </c>
+      <c r="C1028" s="18"/>
+      <c r="D1028" s="18"/>
+      <c r="E1028" s="18" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:5" ht="15" customHeight="1">
+      <c r="A1029" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1029" s="18" t="s">
+        <v>770</v>
+      </c>
+      <c r="C1029" s="18"/>
+      <c r="D1029" s="18"/>
+      <c r="E1029" s="18" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:5" ht="15" customHeight="1">
+      <c r="A1030" s="18" t="s">
+        <v>601</v>
+      </c>
+      <c r="B1030" s="18" t="s">
+        <v>772</v>
+      </c>
+      <c r="C1030" s="18"/>
+      <c r="D1030" s="18"/>
+      <c r="E1030" s="18" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:5" ht="15" customHeight="1">
+      <c r="A1031" s="18"/>
+      <c r="B1031" s="18"/>
+      <c r="C1031" s="18"/>
+      <c r="D1031" s="18"/>
+      <c r="E1031" s="18"/>
     </row>
     <row r="1032" spans="1:5" ht="12.5">
       <c r="A1032" s="4"/>

</xml_diff>

<commit_message>
feat(watchlist): ingest PNP criminality reward snapshot for 2022
</commit_message>
<xml_diff>
--- a/data/rules/pickLists.xlsx
+++ b/data/rules/pickLists.xlsx
@@ -2577,7 +2577,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2628,6 +2628,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -33944,11 +33950,31 @@
       <c r="Z953" s="2"/>
     </row>
     <row r="954" spans="1:26" ht="15" thickBot="1">
-      <c r="A954" s="2"/>
-      <c r="B954" s="2"/>
-      <c r="C954" s="2"/>
-      <c r="D954" s="2"/>
-      <c r="E954" s="2"/>
+      <c r="A954" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sources.ListName</t>
+        </is>
+      </c>
+      <c r="B954" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PNP_MOST_WANTED_WITH_REWARDS_CRIMINALITY_2022</t>
+        </is>
+      </c>
+      <c r="C954" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sources.SourceName</t>
+        </is>
+      </c>
+      <c r="D954" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PNP</t>
+        </is>
+      </c>
+      <c r="E954" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Historical snapshot dated 13 October 2022. Wanted status and reward availability are as listed, not asserted as current.</t>
+        </is>
+      </c>
       <c r="F954" s="2"/>
       <c r="G954" s="2"/>
       <c r="H954" s="2"/>
@@ -33972,11 +33998,23 @@
       <c r="Z954" s="2"/>
     </row>
     <row r="955" spans="1:26" ht="15" thickBot="1">
-      <c r="A955" s="2"/>
-      <c r="B955" s="2"/>
+      <c r="A955" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">additionalInfo.Type</t>
+        </is>
+      </c>
+      <c r="B955" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DILG Memorandum Circular Number</t>
+        </is>
+      </c>
       <c r="C955" s="2"/>
       <c r="D955" s="2"/>
-      <c r="E955" s="2"/>
+      <c r="E955" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DILG circular number as printed in the historical source.</t>
+        </is>
+      </c>
       <c r="F955" s="2"/>
       <c r="G955" s="2"/>
       <c r="H955" s="2"/>
@@ -34000,11 +34038,23 @@
       <c r="Z955" s="2"/>
     </row>
     <row r="956" spans="1:26" ht="15" thickBot="1">
-      <c r="A956" s="2"/>
-      <c r="B956" s="2"/>
+      <c r="A956" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">additionalInfo.Type</t>
+        </is>
+      </c>
+      <c r="B956" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List Reference Date</t>
+        </is>
+      </c>
       <c r="C956" s="2"/>
       <c r="D956" s="2"/>
-      <c r="E956" s="2"/>
+      <c r="E956" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reference date of the source snapshot, not the download date.</t>
+        </is>
+      </c>
       <c r="F956" s="2"/>
       <c r="G956" s="2"/>
       <c r="H956" s="2"/>
@@ -34028,11 +34078,23 @@
       <c r="Z956" s="2"/>
     </row>
     <row r="957" spans="1:26" ht="15" thickBot="1">
-      <c r="A957" s="2"/>
-      <c r="B957" s="2"/>
+      <c r="A957" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">additionalInfo.Type</t>
+        </is>
+      </c>
+      <c r="B957" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identity Note</t>
+        </is>
+      </c>
       <c r="C957" s="2"/>
       <c r="D957" s="2"/>
-      <c r="E957" s="2"/>
+      <c r="E957" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source identity limitations and fallback provenance.</t>
+        </is>
+      </c>
       <c r="F957" s="2"/>
       <c r="G957" s="2"/>
       <c r="H957" s="2"/>

</xml_diff>